<commit_message>
Add dungeon system, combat, AOI, and client network refactor
- Dungeon: DungeonZone, DungeonManager(client), DungeonPortal,
  DungeonEntryPopup, DungeonBot, DungeonData/MapObjectData
- Combat: CombatSystem, MonsterAISystem, combat.proto
  (Attack/Damage/Death/RewardResult/LevelUp), CharacterClassData
- AOI: AoiGrid spatial hash, AoiSystem, InterestComponent,
  SessionSystem refactor for interest-based broadcasting
- Client network: PacketHandler attribute auto-registration,
  partial class handler split (Login/Zone/Entity/Chat/Combat),
  offset-based packet buffer, IL2CPP link.xml
- Zone: base class with HandleMove/HandleChat, CreateSystems virtual
- Data: DataConverter MessagePack array format fix, new data tables
- Bot: multi-account support, DungeonBot for dungeon testing
- DB: 3-database structure (auth/common/game)
- UI: Korean font (NotoSansKR), dungeon entry popup

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/data/xlsx/MonsterData.xlsx
+++ b/server/data/xlsx/MonsterData.xlsx
@@ -1,133 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lemondory/projects/dotnet/data/xlsx/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4C6451-04E2-8B4F-ACFC-E7A639378639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="11540" yWindow="7140" windowWidth="28100" windowHeight="17080" xr2:uid="{91DD000D-CDCF-584E-BD22-924ECBD12A6E}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11540" yWindow="7140" windowWidth="28100" windowHeight="17080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
-  <si>
-    <t>MonsterId</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Hp</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>int</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>ignore</t>
-  </si>
-  <si>
-    <t>몬스터ID</t>
-  </si>
-  <si>
-    <t>이름</t>
-  </si>
-  <si>
-    <t>체력</t>
-  </si>
-  <si>
-    <t>기획 노트</t>
-  </si>
-  <si>
-    <t>작업 상태</t>
-  </si>
-  <si>
-    <t>Slime</t>
-  </si>
-  <si>
-    <t>약한 몬스터</t>
-  </si>
-  <si>
-    <t>완료</t>
-  </si>
-  <si>
-    <t>Goblin</t>
-  </si>
-  <si>
-    <t>중간 몬스터</t>
-  </si>
-  <si>
-    <t>작업중</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="2"/>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
-      <charset val="129"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -143,31 +60,90 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -487,97 +463,485 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35FC2D31-2B52-AA45-9C4E-EAA4B5B3A3D0}">
-  <dimension ref="A1:E5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>MonsterId</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Hp</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>AttackPower</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Defense</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>MoveSpeed</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>AggroRange</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>AttackRange</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>AttackCooldown</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>SkillIds[]</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>SkillIds[]</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ExpReward</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>GoldReward</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MonsterType</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>ignore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>몬스터ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>체력</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>레벨</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>타입</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>공격력</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>방어력</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>이동속도</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>어그로범위(m)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>공격범위(m)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>공격쿨타임(초)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>스킬ID_1</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>스킬ID_2</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>경험치보상</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>골드보상</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Slime</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>약한 슬라임</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Goblin</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L5" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>20</v>
+      </c>
+      <c r="O5" t="n">
+        <v>10</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>기본 고블린</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Orc</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>150</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="N6" t="n">
+        <v>50</v>
+      </c>
+      <c r="O6" t="n">
+        <v>25</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>엘리트 오크</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dragon</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>500</v>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>50</v>
+      </c>
+      <c r="G7" t="n">
+        <v>20</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>15</v>
+      </c>
+      <c r="J7" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4">
+      <c r="K7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" t="n">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4">
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="n">
+        <v>200</v>
+      </c>
+      <c r="O7" t="n">
         <v>100</v>
       </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5">
-        <v>300</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>18</v>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>보스 드래곤</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>